<commit_message>
Mise à jour complète du projet
</commit_message>
<xml_diff>
--- a/data/output_qaqc/qaqc_individus.xlsx
+++ b/data/output_qaqc/qaqc_individus.xlsx
@@ -1,21 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Résumé général" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sexe" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Lien parenté" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Matrimonial" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Niveau études" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Régions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Milieu" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Qualité des données" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Notes méthodologiques" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Résumé général" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sexe" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lien parenté" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrimonial" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Niveau études" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Régions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milieu" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statut emploi" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Secteur activité" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Résidence" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Qualité des données" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes méthodologiques" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -611,7 +614,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>68</t>
         </is>
       </c>
     </row>
@@ -862,6 +865,1524 @@
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>SITUATION DE RÉSIDENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Modalité</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Effectif</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Proportion (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Résident Présent</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>1553511</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>90.72</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Résident Absent</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>116682</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>6.81</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Visiteur</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>42175</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>2.46</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>1,712,368</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>100.00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D71"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>QUALITÉ DES DONNÉES - VALEURS MANQUANTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Nb manquants</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Taux (%)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>niveau_etudes</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>473509</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>27.65</v>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Élevé &gt; 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>niveau_etudes_cm</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>411481</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>24.03</v>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Élevé &gt; 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>handicap_cognitif_brut</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>121388</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>handicap_communication_brut</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>121388</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>handicap_cognitif</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>121388</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>handicap_audition</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>121388</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>handicap_communication</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>121388</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>handicap_moteur</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>121388</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>handicap_audition_brut</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>121388</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>handicap_vision_brut</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>121388</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>handicap_soins_brut</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>121388</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>handicap_moteur_brut</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>121388</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>handicap_vision</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>121388</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>handicap_soins</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>121388</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>alpha_ja</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>alpha_ka</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>alpha_la</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>alpha_nd</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>alpha_ba</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>alpha_br</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>alpha_on</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>alpha_ha</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>alpha_no</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>alpha_mn</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>alpha_sa</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>alpha_gu</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>alpha_pa</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>alpha_by</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>alpha_mj</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>alpha_se</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>alpha_me</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C34" s="4" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>alpha_wy</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>121186</v>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>7.08</v>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Modéré 5–20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>lien_parente</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>39936</v>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>Faible &lt; 5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>situation_matrimoniale_cm</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>39936</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>Faible &lt; 5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>age_cm</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="n">
+        <v>39936</v>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>Faible &lt; 5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>scolarisation_cm</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>39936</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>Faible &lt; 5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>secteur_instit_cm</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="n">
+        <v>39936</v>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>Faible &lt; 5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>statut_emploi_cm</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>39936</v>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>Faible &lt; 5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>taille_menage</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="n">
+        <v>39936</v>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>Faible &lt; 5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>type_menage</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>39936</v>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>Faible &lt; 5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>branche_isic_cm</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="n">
+        <v>39936</v>
+      </c>
+      <c r="C44" s="4" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>Faible &lt; 5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>sexe_cm</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>39936</v>
+      </c>
+      <c r="C45" s="5" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>Faible &lt; 5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>branche_etudes</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="n">
+        <v>38954</v>
+      </c>
+      <c r="C46" s="4" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>Faible &lt; 5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>scolarisation</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>38954</v>
+      </c>
+      <c r="C47" s="5" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>Faible &lt; 5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>departement</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>numind</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="n">
+        <v>69</v>
+      </c>
+      <c r="C50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>men_id</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C51" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>commune</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>milieu_residence</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>situation_residence</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>dept_residence_1an</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>alpha_so</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>alpha_ma</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>alpha_pu</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>alpha_fr</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C59" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D59" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>alpha_wo</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>alpha_ar</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C61" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D61" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>alpha_jo</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D62" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>age</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C63" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>sexe</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C64" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D64" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>region_residence_1an</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C65" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D65" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="18" customHeight="1">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>situation_matrimoniale</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="18" customHeight="1">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>profession</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C67" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D67" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="18" customHeight="1">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>statut_emploi</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D68" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>secteur_instit</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C69" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D69" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="18" customHeight="1">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>branche_isic</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C70" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D70" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>revenu_emploi_estime</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C71" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D71" s="10" t="inlineStr">
+        <is>
+          <t>Complet</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>NOTES MÉTHODOLOGIQUES - DÉCISIONS DE TRAITEMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>TRAITEMENT DES VALEURS ABERRANTES &amp; IMPUTATIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Explication</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Âge (age)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Bornes définies : [0, 120] ans. Imputation par la médiane. Toute valeur hors de ces bornes est corrigée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Variables catégorielles</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Imputation par le mode ou affectation à 'na'/'Unknown' selon les stratégies de config.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>CONTRÔLES DE COHÉRENCE LOGIQUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Explication</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Mariage précoce</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Si l'âge &lt; 12 ans et situation matrimoniale non célibataire, celle-ci est corrigée en 'Célibataire'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Éducation précoce</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Si l'âge &lt; 3 ans et scolarisé, scolarisation est corrigée en 'non, n'a jamais fréquenté'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Sexe et Épouse</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Si sexe différent de Féminin et lien de parenté est Épouse du CM, le sexe est corrigé en 'Féminin'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Travail des enfants</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Si l'âge &lt; 10 ans et statut d'emploi actif (occupé/chômeur), le statut est corrigé en 'Autres inactifs'.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A3:B3"/>
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2145,839 +3666,188 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>QUALITÉ DES DONNÉES - VALEURS MANQUANTES</t>
+          <t>RÉPARTITION PAR STATUT D'EMPLOI</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Variable</t>
+          <t>Modalité</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Nb manquants</t>
+          <t>Effectif</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Taux (%)</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Statut</t>
+          <t>Proportion (%)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>niveau_etudes</t>
+          <t>Autres inactifs</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>473509</v>
+        <v>503183</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>27.65</v>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>Élevé &gt; 20%</t>
-        </is>
+        <v>29.39</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>niveau_etudes_cm</t>
+          <t>Occupé</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>411481</v>
+        <v>343012</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>24.03</v>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>Élevé &gt; 20%</t>
-        </is>
+        <v>20.03</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>alpha_by</t>
+          <t>Etudiant/elève</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>121186</v>
+        <v>298216</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
+        <v>17.42</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>alpha_nd</t>
+          <t>Occupé au foyer</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>121186</v>
+        <v>183340</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
+        <v>10.71</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>alpha_me</t>
+          <t>A la recherche d un premier emploi</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>121186</v>
+        <v>181177</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
+        <v>10.58</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>alpha_ba</t>
+          <t>Autres inactifs, à préciser</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>121186</v>
+        <v>121165</v>
       </c>
       <c r="C9" s="5" t="n">
         <v>7.08</v>
       </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
-      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>alpha_mn</t>
+          <t>Personne du 3e age non pensionnée</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>121186</v>
+        <v>32039</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
+        <v>1.87</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>alpha_no</t>
+          <t>Chômeur ayant travaillé</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>121186</v>
+        <v>20456</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
+        <v>1.19</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>alpha_se</t>
+          <t>Rentier</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>121186</v>
+        <v>18811</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
+        <v>1.1</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>alpha_mj</t>
+          <t>Personne du 3e age pensionnée (FNR ou IPRES)</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>121186</v>
+        <v>10969</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>alpha_br</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="n">
-        <v>121186</v>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>alpha_on</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="n">
-        <v>121186</v>
-      </c>
-      <c r="C15" s="5" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>alpha_pa</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>121186</v>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>alpha_wy</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>121186</v>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>alpha_ka</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="n">
-        <v>121186</v>
-      </c>
-      <c r="C18" s="4" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>alpha_ja</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="n">
-        <v>121186</v>
-      </c>
-      <c r="C19" s="5" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>alpha_gu</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="n">
-        <v>121186</v>
-      </c>
-      <c r="C20" s="4" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>alpha_la</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="n">
-        <v>121186</v>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>alpha_sa</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="n">
-        <v>121186</v>
-      </c>
-      <c r="C22" s="4" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>alpha_ha</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="n">
-        <v>121186</v>
-      </c>
-      <c r="C23" s="5" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>Modéré 5–20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>scolarisation_cm</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="n">
-        <v>39936</v>
-      </c>
-      <c r="C24" s="4" t="n">
-        <v>2.33</v>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>Faible &lt; 5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>age_cm</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>39936</v>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>2.33</v>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>Faible &lt; 5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>lien_parente</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="n">
-        <v>39936</v>
-      </c>
-      <c r="C26" s="4" t="n">
-        <v>2.33</v>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>Faible &lt; 5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>sexe_cm</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="n">
-        <v>39936</v>
-      </c>
-      <c r="C27" s="5" t="n">
-        <v>2.33</v>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>Faible &lt; 5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>situation_matrimoniale_cm</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="n">
-        <v>39936</v>
-      </c>
-      <c r="C28" s="4" t="n">
-        <v>2.33</v>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>Faible &lt; 5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>taille_menage</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="n">
-        <v>39936</v>
-      </c>
-      <c r="C29" s="5" t="n">
-        <v>2.33</v>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
-        <is>
-          <t>Faible &lt; 5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>scolarisation</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="n">
-        <v>38954</v>
-      </c>
-      <c r="C30" s="4" t="n">
-        <v>2.27</v>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>Faible &lt; 5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>branche_etudes</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="n">
-        <v>38954</v>
-      </c>
-      <c r="C31" s="5" t="n">
-        <v>2.27</v>
-      </c>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>Faible &lt; 5%</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>age</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C32" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" s="10" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>commune</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C33" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D33" s="10" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>milieu_residence</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C34" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="10" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>sexe</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C35" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" s="10" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>men_id</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="C36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="10" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>numind</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="n">
-        <v>69</v>
-      </c>
-      <c r="C37" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="10" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>region</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C38" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="10" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>departement</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C39" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" s="10" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>alpha_so</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D40" s="10" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>alpha_pu</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C41" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D41" s="10" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>alpha_wo</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C42" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D42" s="10" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>alpha_fr</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C43" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D43" s="10" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>alpha_ar</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C44" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D44" s="10" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>alpha_ma</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C45" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D45" s="10" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>alpha_jo</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C46" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D46" s="10" t="inlineStr">
-        <is>
-          <t>Complet</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>situation_matrimoniale</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C47" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D47" s="10" t="inlineStr">
-        <is>
-          <t>Complet</t>
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>1,712,368</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>100.00</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2989,135 +3859,123 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>NOTES MÉTHODOLOGIQUES - DÉCISIONS DE TRAITEMENT</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="26" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>TRAITEMENT DES VALEURS ABERRANTES &amp; IMPUTATIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Point</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Explication</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="45" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Âge (age)</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Bornes définies : [0, 120] ans. Imputation par la médiane. Toute valeur hors de ces bornes est corrigée.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Variables catégorielles</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Imputation par le mode ou affectation à 'na'/'Unknown' selon les stratégies de config.py.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>CONTRÔLES DE COHÉRENCE LOGIQUE</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Point</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Explication</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Mariage précoce</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Si l'âge &lt; 12 ans et situation matrimoniale non célibataire, celle-ci est corrigée en 'Célibataire'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Éducation précoce</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Si l'âge &lt; 3 ans et scolarisé, scolarisation est corrigée en 'non, n'a jamais fréquenté'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Sexe et Épouse</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Si sexe différent de Féminin et lien de parenté est Épouse du CM, le sexe est corrigé en 'Féminin'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Travail des enfants</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Si l'âge &lt; 10 ans et statut d'emploi actif (occupé/chômeur), le statut est corrigé en 'Autres inactifs'.</t>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>SECTEUR D'ACTIVITÉ (15 ans et +)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Modalité</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Effectif</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Proportion (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>1369356</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>79.97</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Informel</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>171814</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>10.03</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>111371</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Privé formel</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>59011</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>3.45</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>ISBLSM (ONG, ASC, Fondations, etc.)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>816</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>1,712,368</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>100.00</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A1:B1"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>